<commit_message>
Agrega sugerencias de área desde croquis en la hoja de clasificación
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JxVcM7GXCsdBSUXs7tHjtM
</commit_message>
<xml_diff>
--- a/salida/LIQUIDACION_CONSTRUCCIONES_TIPOLOGIAS_IGAC.xlsx
+++ b/salida/LIQUIDACION_CONSTRUCCIONES_TIPOLOGIAS_IGAC.xlsx
@@ -3794,7 +3794,8 @@
     <comment ref="B11" authorId="0" shapeId="0">
       <text>
         <t>Vida útil vacía en el archivo: se usó la del catálogo (70).
-Área vacía en el archivo (ver croquis en "levantamiento en campo").</t>
+Área vacía en el archivo (ver croquis en "levantamiento en campo").
+SUGERENCIA (no aplicada): Croquis sugiere 7 m × 6,10 m ≈ 42,7 m² ("plataforma carga"); lectura manuscrita dudosa, verificar.</t>
       </text>
     </comment>
     <comment ref="B12" authorId="0" shapeId="0">
@@ -3854,7 +3855,8 @@
     <comment ref="B8" authorId="0" shapeId="0">
       <text>
         <t>Vida útil del archivo (70) distinta a la del catálogo (100); se respetó el archivo.
-Área vacía en el archivo (ver croquis en "levantamiento en campo").</t>
+Área vacía en el archivo (ver croquis en "levantamiento en campo").
+SUGERENCIA (no aplicada): Croquis sugiere comedor de 11 m × 8,80 m ≈ 96,8 m² (el croquis total es 17 m × 8,80 m con baños/oficinas); lectura dudosa, verificar.</t>
       </text>
     </comment>
     <comment ref="B9" authorId="0" shapeId="0">
@@ -22450,7 +22452,7 @@
       </c>
       <c r="O27" s="413" t="inlineStr">
         <is>
-          <t>Vida útil vacía en el archivo: se usó la del catálogo (70). | Área vacía en el archivo (ver croquis en "levantamiento en campo").</t>
+          <t>Vida útil vacía en el archivo: se usó la del catálogo (70). | Área vacía en el archivo (ver croquis en "levantamiento en campo"). | SUGERENCIA (no aplicada): Croquis sugiere 7 m × 6,10 m ≈ 42,7 m² ("plataforma carga"); lectura manuscrita dudosa, verificar.</t>
         </is>
       </c>
       <c r="P27" s="416" t="inlineStr">
@@ -23008,7 +23010,7 @@
       </c>
       <c r="O35" s="422" t="inlineStr">
         <is>
-          <t>Vida útil del archivo (70) distinta a la del catálogo (100); se respetó el archivo. | Área vacía en el archivo (ver croquis en "levantamiento en campo").</t>
+          <t>Vida útil del archivo (70) distinta a la del catálogo (100); se respetó el archivo. | Área vacía en el archivo (ver croquis en "levantamiento en campo"). | SUGERENCIA (no aplicada): Croquis sugiere comedor de 11 m × 8,80 m ≈ 96,8 m² (el croquis total es 17 m × 8,80 m con baños/oficinas); lectura dudosa, verificar.</t>
         </is>
       </c>
       <c r="P35" s="424" t="inlineStr">

</xml_diff>